<commit_message>
Add measurable objectives and key results functionality
- Introduced new SQL script (08_tm_key_results.sql) to create the DCT_TM_KEY_RESULTS table and related structures for managing measurable key results associated with objectives.
- Added lookup vocabularies for key result direction and unit.
- Implemented a new JavaScript component (editDrawer.js) for a slide-in record editor, enhancing the user interface for editing team objectives.
- Included necessary comments and documentation for clarity and future reference.
</commit_message>
<xml_diff>
--- a/final apps/TM/UAT/UAT_TM_TestScript.xlsx
+++ b/final apps/TM/UAT/UAT_TM_TestScript.xlsx
@@ -12,20 +12,22 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross-cutting" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objectives &amp; Key Results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross-cutting" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Access &amp; Session'!$A$1:$I$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dashboard'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Teams'!$A$1:$I$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Team Detail'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Members'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Tasks'!$A$1:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Artifacts'!$A$1:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cross-cutting'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Objectives &amp; Key Results'!$A$1:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Members'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Tasks'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Artifacts'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Cross-cutting'!$A$1:$I$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -514,14 +516,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>• Round 2 · 13-Jun-2026 · Environment: dev-proxy → ADB PROD.</t>
+          <t>• Round 3 · 14-Jun-2026 · Environment: dev-proxy → ADB PROD.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>• Scope: UI/UX rework to the shared platform design + functional enhancements (team edit, member management, task assignment with reassignment tracking, milestones, meetings, documents).</t>
+          <t>• Round 3 focus: measurable objectives (OKR-style Key Results) — per-KR baseline/target/current with auto weighted progress roll-up, a MANUAL override, and full objective + key-result CRUD. Re-runs the full TM regression suite (teams, members, tasks, artifacts, cross-cutting) alongside it.</t>
         </is>
       </c>
     </row>
@@ -542,11 +544,244 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>• Automated results with one evidence screenshot per case: UAT_TM_Results_13-Jun-2026-01.docx.</t>
+          <t>• Automated results with one evidence screenshot per case: UAT_TM_Results_14-Jun-2026-01.docx.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Comments / Defect Ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>TM-XCT-01</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>My Tasks</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Cross-team assigned tasks</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>1. Open My Tasks</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Tasks assigned to me across all teams are listed</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TM-XCT-02</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Management reports catalogue</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>1. Open Reports</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>The management report catalogue renders</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TM-XCT-03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Preferences</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Reminder preferences</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1. Open Preferences
+2. Change lead-days and save</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Lead-days preference saves and persists</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TM-XCT-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>EN ↔ AR RTL</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1. Switch language to Arabic</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Shell flips RTL with Arabic labels; Latin digits retained</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I5"/>
+  <conditionalFormatting sqref="F2:F5">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"PARTIAL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"MANUAL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="F2 F3 F4 F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1282,6 +1517,419 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Test Date</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Comments / Defect Ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-01</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Create objective</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Measurable objective (AUTO)</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>1. Objectives tab → Add Objective
+2. Title + status
+3. Save</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Objective created and listed; progress defaults to AUTO (rolled up from key results)</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-02</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>KR increase</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Add an INCREASE key result</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>1. Open the objective → Add Key Result
+2. Unit %, Increase, baseline 0, target 100, current 50
+3. Save</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>KR shows 50%; the objective auto-progress rolls up to 50%</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>KR decrease + roll-up</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Add a DECREASE key result</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1. Add a second KR: Decrease, baseline 100, target 0, current 75</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>KR shows 25%; the objective weighted roll-up becomes 37.5%</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Update measurement</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Inline current-value update</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1. In the KR row set current = 100
+2. Update</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>The objective auto-progress reflows live to 62.5%</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Manual override</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>MANUAL pins the percentage</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1. Set the objective to Manual at 88%
+2. Change a KR value</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Objective stays 88% (KR changes no longer move it); switch back to Auto restores roll-up</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-06</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Target required</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>KR without a target</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1. Add a KR with no target value</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Rejected with HTTP 400 (boundary)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-07</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Invalid direction</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Bad direction lookup</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>1. Add a KR with an invalid direction</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Rejected with HTTP 400 (lookup validation)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-08</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Permission</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Non-member cannot add a KR</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>1. As a non-member, add a KR</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Denied with HTTP 403 (OBJECTIVE permission)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>TM-OBJ-09</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Delete objective</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Cascade key results</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>1. Remove an objective that has key results</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Objective removed and its key results cascade away</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I10"/>
+  <conditionalFormatting sqref="F2:F10">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"PASS"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"PARTIAL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"MANUAL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1468,276 +2116,6 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="F2 F3 F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Test ID</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Function</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Test Date</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>Comments / Defect Ref</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-01</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Create</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Add a task</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>1. Tasks tab → Add Task
-2. Title, priority, status, due date
-3. Save</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Task created and shown on the Kanban board</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-02</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Kanban move</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Move across columns</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>1. Drag a card to another column (or change status)</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Status changes and status history is written</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Assign</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Assign a member</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Open a task drawer
-2. Assign a team member as primary</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Assignee shown in the drawer with a primary badge</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-04</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Reassign</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Reassignment is tracked</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>1. Set a different member as primary</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Primary moves to the new member AND the activity feed logs the reassignment (audit trail)</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-05</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Activity feed comment</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>1. Post a comment in the task drawer</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Comment appears in the activity feed</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I6"/>
-  <conditionalFormatting sqref="F2:F6">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"PASS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"FAIL"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"PARTIAL"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
-      <formula>"MANUAL"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5 F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1815,27 +2193,29 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-ART-01</t>
+          <t>TM-TSK-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Deliverable</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Add a deliverable</t>
+          <t>Add a task</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Deliverables tab → Add</t>
+          <t>1. Tasks tab → Add Task
+2. Title, priority, status, due date
+3. Save</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Deliverable created and listed</t>
+          <t>Task created and shown on the Kanban board</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1850,27 +2230,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-ART-02</t>
+          <t>TM-TSK-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>RAID</t>
+          <t>Kanban move</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Add a RAID item</t>
+          <t>Move across columns</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. RAID Log tab → Add (Risk, HIGH, OPEN)</t>
+          <t>1. Drag a card to another column (or change status)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>RAID item created and listed</t>
+          <t>Status changes and status history is written</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1885,27 +2265,28 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>TM-ART-03</t>
+          <t>TM-TSK-03</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Milestone</t>
+          <t>Assign</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Add a milestone</t>
+          <t>Assign a member</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>1. Milestones tab → Add (due date, status)</t>
+          <t>1. Open a task drawer
+2. Assign a team member as primary</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Milestone created and listed</t>
+          <t>Assignee shown in the drawer with a primary badge</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1920,27 +2301,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>TM-ART-04</t>
+          <t>TM-TSK-04</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Reassign</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Add a meeting</t>
+          <t>Reassignment is tracked</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1. Meetings tab → Add (date, location, agenda)</t>
+          <t>1. Set a different member as primary</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Meeting created and listed</t>
+          <t>Primary moves to the new member AND the activity feed logs the reassignment (audit trail)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -1955,28 +2336,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>TM-ART-05</t>
+          <t>TM-TSK-05</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>Comment</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Add a team document</t>
+          <t>Activity feed comment</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>1. Documents tab → Add Document
-2. File/name + type + notes</t>
+          <t>1. Post a comment in the task drawer</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Document stored in the unified store (source_module=TM) and listed</t>
+          <t>Comment appears in the activity feed</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -2019,7 +2399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2083,27 +2463,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-01</t>
+          <t>TM-ART-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>My Tasks</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Cross-team assigned tasks</t>
+          <t>Add a deliverable</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Open My Tasks</t>
+          <t>1. Deliverables tab → Add</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Tasks assigned to me across all teams are listed</t>
+          <t>Deliverable created and listed</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -2118,27 +2498,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-02</t>
+          <t>TM-ART-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>RAID</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Management reports catalogue</t>
+          <t>Add a RAID item</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. Open Reports</t>
+          <t>1. RAID Log tab → Add (Risk, HIGH, OPEN)</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>The management report catalogue renders</t>
+          <t>RAID item created and listed</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -2153,28 +2533,27 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-03</t>
+          <t>TM-ART-03</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Preferences</t>
+          <t>Milestone</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Reminder preferences</t>
+          <t>Add a milestone</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>1. Open Preferences
-2. Change lead-days and save</t>
+          <t>1. Milestones tab → Add (due date, status)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Lead-days preference saves and persists</t>
+          <t>Milestone created and listed</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -2189,27 +2568,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-04</t>
+          <t>TM-ART-04</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>EN ↔ AR RTL</t>
+          <t>Add a meeting</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1. Switch language to Arabic</t>
+          <t>1. Meetings tab → Add (date, location, agenda)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Shell flips RTL with Arabic labels; Latin digits retained</t>
+          <t>Meeting created and listed</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -2221,9 +2600,45 @@
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TM-ART-05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Add a team document</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1. Documents tab → Add Document
+2. File/name + type + notes</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Document stored in the unified store (source_module=TM) and listed</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
-  <conditionalFormatting sqref="F2:F5">
+  <autoFilter ref="A1:I6"/>
+  <conditionalFormatting sqref="F2:F6">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2238,7 +2653,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4 F5 F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(atd): add screens for managing subject areas, environments, targets, and queue
- Implemented AtdDiscoveryScreen for subject area discovery with a prompt for new discoveries.
- Created AtdEnvironmentsScreen for full CRUD operations on environments, including a modal for creating/editing.
- Developed AtdTargetsScreen for managing target databases with create/edit functionality.
- Added AtdQueueScreen to display live queue status and actions for reaping stale jobs.
- Introduced AtdRunnerSettingsScreen for editing runner configuration settings with dynamic input fields.
- Added form components (TextField, EnumField, ToggleField) for consistent UI across screens.
</commit_message>
<xml_diff>
--- a/final apps/TM/UAT/UAT_TM_TestScript.xlsx
+++ b/final apps/TM/UAT/UAT_TM_TestScript.xlsx
@@ -8,26 +8,24 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access &amp; Session" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teams" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objectives &amp; Key Results" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Members" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artifacts" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cross-cutting" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Cycle" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive View" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visibility &amp; Security" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Roles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Hierarchy" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Access" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Access &amp; Session'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Dashboard'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Teams'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Team Detail'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Objectives &amp; Key Results'!$A$1:$I$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Members'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Tasks'!$A$1:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Artifacts'!$A$1:$I$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Cross-cutting'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Reporting Cycle'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Executive View'!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Visibility &amp; Security'!$A$1:$I$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Custom Roles'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Team Hierarchy'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'AI Summary'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Timeline'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Access'!$A$1:$I$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -500,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -516,14 +514,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>• Round 3 · 14-Jun-2026 · Environment: dev-proxy → ADB PROD.</t>
+          <t>• Round 4 · 20-Jun-2026 · Environment: dev-proxy → ADB PROD.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>• Round 3 focus: measurable objectives (OKR-style Key Results) — per-KR baseline/target/current with auto weighted progress roll-up, a MANUAL override, and full objective + key-result CRUD. Re-runs the full TM regression suite (teams, members, tasks, artifacts, cross-cutting) alongside it.</t>
+          <t>• Round 4 focus: the Reporting-Cycle wave — periodic reporting cycles + member check-ins, the cross-DCT executive view (scorecard + achievement badges), cross-team visibility grants (executive exceptions) and the row-level security retrofit, admin custom-role CRUD, parent-child team hierarchy, the AI period summary, and the Gantt/timeline view.</t>
         </is>
       </c>
     </row>
@@ -537,14 +535,21 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>• Status legend: PASS / FAIL / PARTIAL / MANUAL / SKIP (Status column has a dropdown).</t>
+          <t>• Security cases prove a team cannot see another team’s data unless an explicit grant applies.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>• Automated results with one evidence screenshot per case: UAT_TM_Results_14-Jun-2026-01.docx.</t>
+          <t>• Status legend: PASS / FAIL / PARTIAL / MANUAL / SKIP (Status column has a dropdown).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>• Automated results with one evidence screenshot per case: UAT_TM_Results_20-Jun-2026-02.docx.</t>
         </is>
       </c>
     </row>
@@ -553,17 +558,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -623,27 +628,29 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-01</t>
+          <t>TM-CYC-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>My Tasks</t>
+          <t>Cadence config</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Cross-team assigned tasks</t>
+          <t>Save a reporting cadence</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Open My Tasks</t>
+          <t>1. Open a team’s Reporting Cycle
+2. Set Monthly, ALL_MEMBERS, lead 3d, reminders 3,1
+3. Save</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Tasks assigned to me across all teams are listed</t>
+          <t>Cadence saved and rendered on the Reporting Cycle page</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -658,27 +665,29 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-02</t>
+          <t>TM-CYC-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Generate periods</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Management reports catalogue</t>
+          <t>Generate + idempotency</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. Open Reports</t>
+          <t>1. Save a cadence
+2. Generate periods
+3. Generate again</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>The management report catalogue renders</t>
+          <t>Periods generated through the horizon; a second generate adds 0 (idempotent)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -693,28 +702,29 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-03</t>
+          <t>TM-CYC-03</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Preferences</t>
+          <t>Member check-in (draft)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Reminder preferences</t>
+          <t>Member saves a draft</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>1. Open Preferences
-2. Change lead-days and save</t>
+          <t>1. As a member, open My Check-ins
+2. Fill the narrative fields
+3. Save Draft</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Lead-days preference saves and persists</t>
+          <t>Draft saved and listed in My Check-ins with auto-pulled metrics</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -729,27 +739,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>TM-XCT-04</t>
+          <t>TM-CYC-04</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Language</t>
+          <t>Check-in modal</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>EN ↔ AR RTL</t>
+          <t>Narrative + auto-metrics</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1. Switch language to Arabic</t>
+          <t>1. Open the check-in row</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Shell flips RTL with Arabic labels; Latin digits retained</t>
+          <t>Modal shows narrative fields + read-only auto-metric tiles (tasks done/late/overdue, KPI)</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -761,9 +771,220 @@
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr"/>
     </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TM-CYC-05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Member submit</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>On-time submission</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1. Submit the check-in before the due date</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Status becomes SUBMITTED (or LATE past due) — evaluated server-side</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>TM-CYC-06</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Leader roster</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Period status roster</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1. As leader, open the period roster</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Roster lists each submitter with status + metrics; the member shows SUBMITTED</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>TM-CYC-07</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Leader sign-off</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Sign off with RAG</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>1. Set team RAG + summary
+2. Sign off</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Sign-off (RAG + summary) stored on the period</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>TM-CYC-08</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Close + snapshot</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Immutable snapshot</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>1. Close the period</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Close writes a well-formed, immutable JSON snapshot; status → CLOSED</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>TM-CYC-09</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Closed is read-only</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Edit a closed period</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>1. As a member, try to edit a CLOSED period</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Rejected with HTTP 400 (period closed; immutability)</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>TM-CYC-10</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Lock period</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Freeze the record</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>1. Lock the closed period</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Status → LOCKED (record frozen)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I5"/>
-  <conditionalFormatting sqref="F2:F5">
+  <autoFilter ref="A1:I11"/>
+  <conditionalFormatting sqref="F2:F11">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -778,207 +999,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="40" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Test ID</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Function</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Tested By</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Test Date</t>
-        </is>
-      </c>
-      <c r="I1" s="3" t="inlineStr">
-        <is>
-          <t>Comments / Defect Ref</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>TM-ACC-01</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Shared session</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Entry from Admin via switcher</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>1. Login in the Admin app
-2. Open the module switcher
-3. Choose Task Management</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>TM (App 207) opens logged-in with no second login; TM brand cube; role-appropriate nav</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>TM-ACC-02</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>No session</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Direct open without login</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>1. Logout / fresh private window
-2. Open the TM app URL directly</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Redirected to the Admin portal login; no TM content before login</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TM-ACC-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Role gating</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Admin-only nav hidden for non-admin</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Enter TM as a non-admin user</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Team Roles (admin) nav hidden for non-admins; Teams/My Tasks available</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I4"/>
-  <conditionalFormatting sqref="F2:F4">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"PASS"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"FAIL"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
-      <formula>"PARTIAL"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
-      <formula>"MANUAL"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10 F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -992,11 +1013,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -1056,27 +1077,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-DSH-01</t>
+          <t>TM-EXE-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>KPI tiles</t>
+          <t>Render</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Five live KPI tiles</t>
+          <t>Roll-up KPIs + charts + scorecard</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Open the TM dashboard</t>
+          <t>1. Open the Executive view</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>My Teams / My Open Tasks / Overdue / Open Issues &amp; Risks / Deliverables Due tiles show live numbers</t>
+          <t>4 roll-up KPIs, RAG + on-time charts, and the team scorecard render</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1091,27 +1112,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-DSH-02</t>
+          <t>TM-EXE-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Charts</t>
+          <t>Group by</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Teams by Health + Class</t>
+          <t>Org / team-tree / flat</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. Open the dashboard and wait for charts</t>
+          <t>1. Toggle the Group-by selector</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Both Chart.js charts render with data (no empty boxes)</t>
+          <t>The scorecard regroups by org node, by team hierarchy, and flat</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1123,9 +1144,79 @@
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TM-EXE-03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Scorecard API</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Full performance metrics</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1. Inspect exec/teams</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Each visible team returns tasks done/overdue, risks, objective %, and on-time rate</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TM-EXE-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Badges</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Achievement badges</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1. Inspect the scorecard for badge eligibility</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Teams qualify for zero-overdue / perfect on-time / all-on-track badges</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
-  <conditionalFormatting sqref="F2:F3">
+  <autoFilter ref="A1:I5"/>
+  <conditionalFormatting sqref="F2:F5">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1140,7 +1231,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4 F5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1154,11 +1245,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -1218,27 +1309,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-TMS-01</t>
+          <t>TM-SEC-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>List</t>
+          <t>Member scope (list)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Team grid loads</t>
+          <t>Other teams hidden</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Open Teams</t>
+          <t>1. As a member, list teams</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Team cards show code, health RAG, type/class and member/task counts</t>
+          <t>A team the member does not belong to is NOT in their list (row-level scope)</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1253,27 +1344,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-TMS-02</t>
+          <t>TM-SEC-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Filter</t>
+          <t>Member scope (detail)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Type/class/status filters</t>
+          <t>Other team detail denied</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. On Teams pick a Type filter</t>
+          <t>1. As a member, open a non-member team</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Grid re-queries server-side and shows matching teams</t>
+          <t>Denied with HTTP 403/404 (visibility guard)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1288,29 +1379,27 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>TM-TMS-03</t>
+          <t>TM-SEC-03</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Create</t>
+          <t>Grant create</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>New team via platform modal</t>
+          <t>Executive exception</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>1. Teams → New Team
-2. Fill name, type, class, objective
-3. Create</t>
+          <t>1. As admin, grant the member VIEWER access to the team</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Team created with a TM- code; creator auto-enrolled as Leader; appears in the grid</t>
+          <t>Grant created ACTIVE and listed</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1322,9 +1411,80 @@
       <c r="H4" s="4" t="inlineStr"/>
       <c r="I4" s="4" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>TM-SEC-04</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Grant exposes</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Exception takes effect</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1. As the member, read the granted team</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>The member can now read the team (detail 200 + appears in their list)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TM-SEC-05</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Grant revoke</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Exception removed</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1. As admin, revoke the grant
+2. As the member, read the team</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>The team is immediately re-hidden (HTTP 403/404)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
-  <conditionalFormatting sqref="F2:F4">
+  <autoFilter ref="A1:I6"/>
+  <conditionalFormatting sqref="F2:F6">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1339,7 +1499,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4 F5 F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1353,11 +1513,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -1417,27 +1577,29 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-DTL-01</t>
+          <t>TM-ROL-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Create role</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Full team definition grid</t>
+          <t>Admin custom role</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Open a team</t>
+          <t>1. Team Roles → New Role
+2. Code/name/leader flag
+3. Save</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Overview shows ALL team fields in an aligned definition grid + KPI tiles + 9 tabs</t>
+          <t>Custom team-role created and present in the role list</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1452,29 +1614,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-DTL-02</t>
+          <t>TM-ROL-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Edit team</t>
+          <t>Edit matrix</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Edit Team modal persists</t>
+          <t>Template CRUD matrix</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. Open a team → Edit Team
-2. Change objective + status
-3. Save Changes</t>
+          <t>1. Toggle the artifact CRUD cells for the role</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Edit modal (top-right) saves via PUT; changes persist on reload</t>
+          <t>Template permission defaults updated (e.g. TASK = C/R/U, no Delete)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1486,9 +1646,44 @@
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
     </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>TM-ROL-03</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Retire role</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Retire a custom role</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1. Retire the custom role</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Custom role retired; built-in (is_system) roles stay protected</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
+      <c r="H4" s="4" t="inlineStr"/>
+      <c r="I4" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
-  <conditionalFormatting sqref="F2:F3">
+  <autoFilter ref="A1:I4"/>
+  <conditionalFormatting sqref="F2:F4">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1503,7 +1698,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3 F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1517,11 +1712,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -1581,29 +1776,28 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-OBJ-01</t>
+          <t>TM-HIER-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Create objective</t>
+          <t>Set parent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Measurable objective (AUTO)</t>
+          <t>Parent-child link</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Objectives tab → Add Objective
-2. Title + status
-3. Save</t>
+          <t>1. Re-parent a team under another
+2. Check the team-tree</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Objective created and listed; progress defaults to AUTO (rolled up from key results)</t>
+          <t>The child team shows the new parent in the team-tree</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1618,29 +1812,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-OBJ-02</t>
+          <t>TM-HIER-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>KR increase</t>
+          <t>Cycle guard</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Add an INCREASE key result</t>
+          <t>Reject a parent cycle</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. Open the objective → Add Key Result
-2. Unit %, Increase, baseline 0, target 100, current 50
-3. Save</t>
+          <t>1. Try to make the parent a child of its own descendant</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>KR shows 50%; the objective auto-progress rolls up to 50%</t>
+          <t>Rejected with HTTP 400 (cycle guard)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1652,256 +1844,9 @@
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>KR decrease + roll-up</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Add a DECREASE key result</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Add a second KR: Decrease, baseline 100, target 0, current 75</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>KR shows 25%; the objective weighted roll-up becomes 37.5%</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-04</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Update measurement</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Inline current-value update</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>1. In the KR row set current = 100
-2. Update</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>The objective auto-progress reflows live to 62.5%</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-05</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Manual override</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>MANUAL pins the percentage</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>1. Set the objective to Manual at 88%
-2. Change a KR value</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Objective stays 88% (KR changes no longer move it); switch back to Auto restores roll-up</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-06</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Target required</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>KR without a target</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>1. Add a KR with no target value</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Rejected with HTTP 400 (boundary)</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
-      <c r="I7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-07</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Invalid direction</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Bad direction lookup</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>1. Add a KR with an invalid direction</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Rejected with HTTP 400 (lookup validation)</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
-      <c r="I8" s="4" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-08</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Permission</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Non-member cannot add a KR</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>1. As a non-member, add a KR</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Denied with HTTP 403 (OBJECTIVE permission)</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
-      <c r="I9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>TM-OBJ-09</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Delete objective</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Cascade key results</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>1. Remove an objective that has key results</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Objective removed and its key results cascade away</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I10"/>
-  <conditionalFormatting sqref="F2:F10">
+  <autoFilter ref="A1:I3"/>
+  <conditionalFormatting sqref="F2:F3">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -1916,7 +1861,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5 F6 F7 F8 F9 F10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1930,11 +1875,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -1994,29 +1939,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-MBR-01</t>
+          <t>TM-AI-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Add member</t>
+          <t>Generate</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Add from the user picker</t>
+          <t>AI period summary</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Members tab → Add Member
-2. Pick a user + role + title
-3. Add</t>
+          <t>1. As leader/admin, generate the AI summary for a period</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Member added from DCT_USERS and listed with avatar + role</t>
+          <t>A board-ready narrative is generated from the period data and stored</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -2031,27 +1974,27 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>TM-MBR-02</t>
+          <t>TM-AI-02</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Change role</t>
+          <t>Permission</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Inline role change</t>
+          <t>Non-viewer denied</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1. Change a member’s role in the row dropdown</t>
+          <t>1. As a non-viewer, read another team’s AI summary</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>New team role persists</t>
+          <t>Denied with HTTP 403/404</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -2063,44 +2006,9 @@
       <c r="H3" s="4" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TM-MBR-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Remove member</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Remove from team</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Click remove on a member row</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Member removed and no longer listed</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I4"/>
-  <conditionalFormatting sqref="F2:F4">
+  <autoFilter ref="A1:I3"/>
+  <conditionalFormatting sqref="F2:F3">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2115,7 +2023,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2 F3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2129,11 +2037,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -2193,29 +2101,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-TSK-01</t>
+          <t>TM-TL-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Create</t>
+          <t>Gantt render</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Add a task</t>
+          <t>Timeline view</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Tasks tab → Add Task
-2. Title, priority, status, due date
-3. Save</t>
+          <t>1. Open a team’s Timeline</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Task created and shown on the Kanban board</t>
+          <t>A month axis + bars for tasks/deliverables/milestones render</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -2227,150 +2133,9 @@
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="4" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-02</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Kanban move</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Move across columns</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>1. Drag a card to another column (or change status)</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Status changes and status history is written</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Assign</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Assign a member</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Open a task drawer
-2. Assign a team member as primary</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Assignee shown in the drawer with a primary badge</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-04</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Reassign</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Reassignment is tracked</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>1. Set a different member as primary</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Primary moves to the new member AND the activity feed logs the reassignment (audit trail)</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>TM-TSK-05</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Comment</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Activity feed comment</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>1. Post a comment in the task drawer</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Comment appears in the activity feed</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
-  <conditionalFormatting sqref="F2:F6">
+  <autoFilter ref="A1:I2"/>
+  <conditionalFormatting sqref="F2">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2385,7 +2150,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5 F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2399,11 +2164,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
@@ -2463,27 +2228,27 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>TM-ART-01</t>
+          <t>TM-ACC-01</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Deliverable</t>
+          <t>Member nav</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Add a deliverable</t>
+          <t>Role-appropriate nav</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>1. Deliverables tab → Add</t>
+          <t>1. Enter TM as a non-admin</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Deliverable created and listed</t>
+          <t>My Check-ins is available; admin-only Visibility/Roles nav is hidden</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -2495,150 +2260,9 @@
       <c r="H2" s="4" t="inlineStr"/>
       <c r="I2" s="4" t="inlineStr"/>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>TM-ART-02</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>RAID</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Add a RAID item</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>1. RAID Log tab → Add (Risk, HIGH, OPEN)</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>RAID item created and listed</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
-      <c r="I3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>TM-ART-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Milestone</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Add a milestone</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>1. Milestones tab → Add (due date, status)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Milestone created and listed</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
-      <c r="I4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>TM-ART-04</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Meeting</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Add a meeting</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>1. Meetings tab → Add (date, location, agenda)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Meeting created and listed</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>TM-ART-05</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Document</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Add a team document</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>1. Documents tab → Add Document
-2. File/name + type + notes</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Document stored in the unified store (source_module=TM) and listed</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
-      <c r="I6" s="4" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I6"/>
-  <conditionalFormatting sqref="F2:F6">
+  <autoFilter ref="A1:I2"/>
+  <conditionalFormatting sqref="F2">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"PASS"</formula>
     </cfRule>
@@ -2653,7 +2277,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F2 F3 F4 F5 F6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,PARTIAL,MANUAL,SKIP,Not Run"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>